<commit_message>
Fix priority coloring with conditional formatting
</commit_message>
<xml_diff>
--- a/Pending_Tasks_Tracker.xlsx
+++ b/Pending_Tasks_Tracker.xlsx
@@ -43,7 +43,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -67,22 +67,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -132,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -146,9 +131,24 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -158,6 +158,15 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -167,28 +176,98 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="8">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="009C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="009C6500"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="00006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="001F4E78"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00BDD7EE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="009C6500"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="00808080"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="009C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -684,7 +763,7 @@
           <t>Layout / Fit-out</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -736,354 +815,354 @@
       <c r="K5" s="4" t="inlineStr"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="7" t="n">
+      <c r="A6" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Central 50</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>Tank fitting on coffee</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>Equipment / Plumbing</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G6" s="8" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr"/>
-      <c r="I6" s="7" t="inlineStr"/>
-      <c r="J6" s="7" t="inlineStr"/>
-      <c r="K6" s="8" t="inlineStr"/>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="6" t="inlineStr"/>
+      <c r="I6" s="6" t="inlineStr"/>
+      <c r="J6" s="6" t="inlineStr"/>
+      <c r="K6" s="7" t="inlineStr"/>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Central 50</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Misting fans repair</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Repair / Maintenance</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G7" s="8" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr"/>
-      <c r="I7" s="7" t="inlineStr"/>
-      <c r="J7" s="7" t="inlineStr"/>
-      <c r="K7" s="8" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="inlineStr"/>
+      <c r="K7" s="7" t="inlineStr"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="7" t="n">
+      <c r="A8" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Central 50</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>Covers for furniture</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>Procurement</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G8" s="8" t="inlineStr"/>
-      <c r="H8" s="7" t="inlineStr"/>
-      <c r="I8" s="7" t="inlineStr"/>
-      <c r="J8" s="7" t="inlineStr"/>
-      <c r="K8" s="8" t="inlineStr"/>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr"/>
+      <c r="H8" s="6" t="inlineStr"/>
+      <c r="I8" s="6" t="inlineStr"/>
+      <c r="J8" s="6" t="inlineStr"/>
+      <c r="K8" s="7" t="inlineStr"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>Central 50</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Sahil signages repair work</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>Signage / Repair</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="inlineStr"/>
-      <c r="H9" s="7" t="inlineStr"/>
-      <c r="I9" s="7" t="inlineStr"/>
-      <c r="J9" s="7" t="inlineStr"/>
-      <c r="K9" s="8" t="inlineStr"/>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr"/>
+      <c r="H9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="inlineStr"/>
+      <c r="K9" s="7" t="inlineStr"/>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="7" t="n">
+      <c r="A10" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Central 50</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>Plantation for aesthetic beautification</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>Landscaping / Aesthetics</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G10" s="8" t="inlineStr"/>
-      <c r="H10" s="7" t="inlineStr"/>
-      <c r="I10" s="7" t="inlineStr"/>
-      <c r="J10" s="7" t="inlineStr"/>
-      <c r="K10" s="8" t="inlineStr"/>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr"/>
+      <c r="H10" s="6" t="inlineStr"/>
+      <c r="I10" s="6" t="inlineStr"/>
+      <c r="J10" s="6" t="inlineStr"/>
+      <c r="K10" s="7" t="inlineStr"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Central 50</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Taps of Heaven deal closure</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>Business / Deal</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G11" s="8" t="inlineStr"/>
-      <c r="H11" s="7" t="inlineStr"/>
-      <c r="I11" s="7" t="inlineStr"/>
-      <c r="J11" s="7" t="inlineStr"/>
-      <c r="K11" s="8" t="inlineStr"/>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr"/>
+      <c r="H11" s="6" t="inlineStr"/>
+      <c r="I11" s="6" t="inlineStr"/>
+      <c r="J11" s="6" t="inlineStr"/>
+      <c r="K11" s="7" t="inlineStr"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="7" t="n">
+      <c r="A12" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Central 50</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>D Kitchen deadline</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>Kitchen / Operations</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G12" s="8" t="inlineStr"/>
-      <c r="H12" s="7" t="inlineStr"/>
-      <c r="I12" s="7" t="inlineStr"/>
-      <c r="J12" s="7" t="inlineStr"/>
-      <c r="K12" s="8" t="inlineStr"/>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr"/>
+      <c r="H12" s="6" t="inlineStr"/>
+      <c r="I12" s="6" t="inlineStr"/>
+      <c r="J12" s="6" t="inlineStr"/>
+      <c r="K12" s="7" t="inlineStr"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="10" t="n">
+      <c r="A13" s="9" t="n">
         <v>11</v>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Bennett University</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>Electrical connections - all brands</t>
         </is>
       </c>
-      <c r="D13" s="11" t="inlineStr">
+      <c r="D13" s="10" t="inlineStr">
         <is>
           <t>Electrical</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E13" s="11" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F13" s="10" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G13" s="11" t="inlineStr"/>
-      <c r="H13" s="10" t="inlineStr"/>
-      <c r="I13" s="10" t="inlineStr"/>
-      <c r="J13" s="10" t="inlineStr"/>
-      <c r="K13" s="11" t="inlineStr"/>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr"/>
+      <c r="H13" s="9" t="inlineStr"/>
+      <c r="I13" s="9" t="inlineStr"/>
+      <c r="J13" s="9" t="inlineStr"/>
+      <c r="K13" s="10" t="inlineStr"/>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="10" t="n">
+      <c r="A14" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Bennett University</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>Water connections - all brands</t>
         </is>
       </c>
-      <c r="D14" s="11" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>Plumbing / Water</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F14" s="10" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G14" s="11" t="inlineStr"/>
-      <c r="H14" s="10" t="inlineStr"/>
-      <c r="I14" s="10" t="inlineStr"/>
-      <c r="J14" s="10" t="inlineStr"/>
-      <c r="K14" s="11" t="inlineStr"/>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr"/>
+      <c r="H14" s="9" t="inlineStr"/>
+      <c r="I14" s="9" t="inlineStr"/>
+      <c r="J14" s="9" t="inlineStr"/>
+      <c r="K14" s="10" t="inlineStr"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="10" t="n">
+      <c r="A15" s="9" t="n">
         <v>13</v>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Bennett University</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>Grease trap</t>
         </is>
       </c>
-      <c r="D15" s="11" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>Plumbing / Kitchen</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E15" s="11" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F15" s="10" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G15" s="11" t="inlineStr"/>
-      <c r="H15" s="10" t="inlineStr"/>
-      <c r="I15" s="10" t="inlineStr"/>
-      <c r="J15" s="10" t="inlineStr"/>
-      <c r="K15" s="11" t="inlineStr"/>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr"/>
+      <c r="H15" s="9" t="inlineStr"/>
+      <c r="I15" s="9" t="inlineStr"/>
+      <c r="J15" s="9" t="inlineStr"/>
+      <c r="K15" s="10" t="inlineStr"/>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="12" t="n">
@@ -1104,7 +1183,7 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="E16" s="14" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -1121,80 +1200,108 @@
       <c r="K16" s="13" t="inlineStr"/>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="14" t="n">
+      <c r="A17" s="15" t="n">
         <v>15</v>
       </c>
-      <c r="B17" s="15" t="inlineStr">
+      <c r="B17" s="16" t="inlineStr">
         <is>
           <t>Sector 1 Noida</t>
         </is>
       </c>
-      <c r="C17" s="15" t="inlineStr">
+      <c r="C17" s="16" t="inlineStr">
         <is>
           <t>Awaiting tasks - to be added</t>
         </is>
       </c>
-      <c r="D17" s="15" t="inlineStr">
+      <c r="D17" s="16" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E17" s="17" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F17" s="14" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G17" s="15" t="inlineStr"/>
-      <c r="H17" s="14" t="inlineStr"/>
-      <c r="I17" s="14" t="inlineStr"/>
-      <c r="J17" s="14" t="inlineStr"/>
-      <c r="K17" s="15" t="inlineStr"/>
+      <c r="F17" s="15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr"/>
+      <c r="H17" s="15" t="inlineStr"/>
+      <c r="I17" s="15" t="inlineStr"/>
+      <c r="J17" s="15" t="inlineStr"/>
+      <c r="K17" s="16" t="inlineStr"/>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="16" t="n">
+      <c r="A18" s="18" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="17" t="inlineStr">
+      <c r="B18" s="19" t="inlineStr">
         <is>
           <t>General</t>
         </is>
       </c>
-      <c r="C18" s="17" t="inlineStr">
+      <c r="C18" s="19" t="inlineStr">
         <is>
           <t>ETL housekeeping uniforms</t>
         </is>
       </c>
-      <c r="D18" s="17" t="inlineStr">
+      <c r="D18" s="19" t="inlineStr">
         <is>
           <t>Housekeeping / Procurement</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="E18" s="20" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F18" s="16" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G18" s="17" t="inlineStr"/>
-      <c r="H18" s="16" t="inlineStr"/>
-      <c r="I18" s="16" t="inlineStr"/>
-      <c r="J18" s="16" t="inlineStr"/>
-      <c r="K18" s="17" t="inlineStr"/>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G18" s="19" t="inlineStr"/>
+      <c r="H18" s="18" t="inlineStr"/>
+      <c r="I18" s="18" t="inlineStr"/>
+      <c r="J18" s="18" t="inlineStr"/>
+      <c r="K18" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:K18"/>
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>
   </mergeCells>
+  <conditionalFormatting sqref="E3:E18">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"High"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"Medium"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"Low"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F3:F18">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+      <formula>"Completed"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
+      <formula>"In Progress"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="5">
+      <formula>"On Hold"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="6">
+      <formula>"Cancelled"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="7">
+      <formula>"Pending"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation sqref="E3:E18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"High,Medium,Low"</formula1>

</xml_diff>

<commit_message>
Add District 9 tasks to tracker
</commit_message>
<xml_diff>
--- a/Pending_Tasks_Tracker.xlsx
+++ b/Pending_Tasks_Tracker.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Task Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Task Tracker'!$A$2:$K$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Task Tracker'!$A$2:$K$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -629,7 +629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1170,22 +1170,22 @@
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>D9</t>
+          <t>District 9</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
         <is>
-          <t>Awaiting tasks - to be added</t>
+          <t>ETL signages - entry</t>
         </is>
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Signage</t>
         </is>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F16" s="12" t="inlineStr">
@@ -1200,81 +1200,151 @@
       <c r="K16" s="13" t="inlineStr"/>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="15" t="n">
+      <c r="A17" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="B17" s="16" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>District 9</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>ETL signages - lamps</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>Signage / Lighting</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G17" s="13" t="inlineStr"/>
+      <c r="H17" s="12" t="inlineStr"/>
+      <c r="I17" s="12" t="inlineStr"/>
+      <c r="J17" s="12" t="inlineStr"/>
+      <c r="K17" s="13" t="inlineStr"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>District 9</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>New furniture</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Procurement</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G18" s="13" t="inlineStr"/>
+      <c r="H18" s="12" t="inlineStr"/>
+      <c r="I18" s="12" t="inlineStr"/>
+      <c r="J18" s="12" t="inlineStr"/>
+      <c r="K18" s="13" t="inlineStr"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
         <is>
           <t>Sector 1 Noida</t>
         </is>
       </c>
-      <c r="C17" s="16" t="inlineStr">
+      <c r="C19" s="16" t="inlineStr">
         <is>
           <t>Awaiting tasks - to be added</t>
         </is>
       </c>
-      <c r="D17" s="16" t="inlineStr">
+      <c r="D19" s="16" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="E17" s="17" t="inlineStr">
+      <c r="E19" s="17" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F17" s="15" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G17" s="16" t="inlineStr"/>
-      <c r="H17" s="15" t="inlineStr"/>
-      <c r="I17" s="15" t="inlineStr"/>
-      <c r="J17" s="15" t="inlineStr"/>
-      <c r="K17" s="16" t="inlineStr"/>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="18" t="n">
-        <v>16</v>
-      </c>
-      <c r="B18" s="19" t="inlineStr">
+      <c r="F19" s="15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr"/>
+      <c r="H19" s="15" t="inlineStr"/>
+      <c r="I19" s="15" t="inlineStr"/>
+      <c r="J19" s="15" t="inlineStr"/>
+      <c r="K19" s="16" t="inlineStr"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="18" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="19" t="inlineStr">
         <is>
           <t>General</t>
         </is>
       </c>
-      <c r="C18" s="19" t="inlineStr">
+      <c r="C20" s="19" t="inlineStr">
         <is>
           <t>ETL housekeeping uniforms</t>
         </is>
       </c>
-      <c r="D18" s="19" t="inlineStr">
+      <c r="D20" s="19" t="inlineStr">
         <is>
           <t>Housekeeping / Procurement</t>
         </is>
       </c>
-      <c r="E18" s="20" t="inlineStr">
+      <c r="E20" s="20" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F18" s="18" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G18" s="19" t="inlineStr"/>
-      <c r="H18" s="18" t="inlineStr"/>
-      <c r="I18" s="18" t="inlineStr"/>
-      <c r="J18" s="18" t="inlineStr"/>
-      <c r="K18" s="19" t="inlineStr"/>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G20" s="19" t="inlineStr"/>
+      <c r="H20" s="18" t="inlineStr"/>
+      <c r="I20" s="18" t="inlineStr"/>
+      <c r="J20" s="18" t="inlineStr"/>
+      <c r="K20" s="19" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:K18"/>
+  <autoFilter ref="A2:K20"/>
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>
   </mergeCells>
-  <conditionalFormatting sqref="E3:E18">
+  <conditionalFormatting sqref="E3:E20">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"High"</formula>
     </cfRule>
@@ -1285,7 +1355,7 @@
       <formula>"Low"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F3:F18">
+  <conditionalFormatting sqref="F3:F20">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"Completed"</formula>
     </cfRule>
@@ -1303,10 +1373,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="E3:E18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E3:E20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation sqref="F3:F18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F3:F20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,In Progress,On Hold,Completed,Cancelled"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>